<commit_message>
ver -2116 賽西莉差分 11 張＋愛里歐 hurtsmile 接線（美術 441ba93c）；pant 跪姿 cm/standCm 估值；lint 例外 cecilie.nosebleed；重出差分總表
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/si/_SI_差分總表.xlsx
+++ b/resources/si/_SI_差分總表.xlsx
@@ -19676,42 +19676,47 @@
       </c>
     </row>
     <row r="6" ht="111" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>謎之術師</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>mage_si_hurtsmile.webp</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="n"/>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>hurtsmile</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>1529</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>resources/si/npc/mage_si_hurtsmile.webp</t>
         </is>
@@ -31145,7 +31150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D151"/>
+  <dimension ref="A1:D139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -31272,12 +31277,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>image - 2026-09-26T205756.614</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cecilie_si_battlecry.webp</t>
+          <t>image - 2026-09-26T205756.614.png</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -31294,12 +31299,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cecilie_si_call.webp</t>
+          <t>luna_si_front.webp</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -31316,12 +31321,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>cecilie_si_command.webp</t>
+          <t>luna_si_seat_lookdown.webp</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -31338,12 +31343,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle_nun</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>cecilie_si_nosebleed.webp</t>
+          <t>nouvelle_nun_si_front.webp</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -31360,12 +31365,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>cecilie_si_pant.webp</t>
+          <t>nouvelle_si_back.webp</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -31382,12 +31387,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>cecilie_si_proud.webp</t>
+          <t>nouvelle_si_bye.webp</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -31404,12 +31409,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>cecilie_si_ready.webp</t>
+          <t>nouvelle_si_expainsweat.webp</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -31426,12 +31431,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>cecilie_si_shocknose.webp</t>
+          <t>nouvelle_si_meetagain.webp</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -31448,12 +31453,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>cecilie_si_shyhand.webp</t>
+          <t>nouvelle_si_reliefbreath.webp</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -31470,12 +31475,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>cecilie_si_shynose.webp</t>
+          <t>nouvelle_si_scare.webp</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -31492,12 +31497,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>cecilie_si_smirk.webp</t>
+          <t>nouvelle_si_side.webp</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -31514,12 +31519,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>image - 2026-09-26T205756.614</t>
+          <t>Npc_aaron</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>image - 2026-09-26T205756.614.png</t>
+          <t>npc_aaron_si_trial.png</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -31536,12 +31541,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Luna</t>
+          <t>Npc_molly</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>luna_si_front.webp</t>
+          <t>npc_molly_si_trial.png</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -31558,12 +31563,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Luna</t>
+          <t>Npc_robert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>luna_si_seat_lookdown.webp</t>
+          <t>npc_robert_si_trial.png</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -31580,12 +31585,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nouvelle_nun</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>nouvelle_nun_si_front.webp</t>
+          <t>aaron_si_angry.webp</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -31602,12 +31607,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>nouvelle_si_back.webp</t>
+          <t>aaron_si_armscross.webp</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -31624,12 +31629,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>nouvelle_si_bye.webp</t>
+          <t>aaron_si_attention.webp</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -31646,12 +31651,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>nouvelle_si_expainsweat.webp</t>
+          <t>aaron_si_blindeye.webp</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -31668,12 +31673,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>nouvelle_si_meetagain.webp</t>
+          <t>aaron_si_closedsmile.webp</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -31690,12 +31695,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>nouvelle_si_reliefbreath.webp</t>
+          <t>aaron_si_confused.webp</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -31712,12 +31717,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>nouvelle_si_scare.webp</t>
+          <t>aaron_si_draw.webp</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -31734,12 +31739,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>nouvelle_si_side.webp</t>
+          <t>aaron_si_front.webp</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -31756,12 +31761,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Npc_aaron</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>npc_aaron_si_trial.png</t>
+          <t>aaron_si_signal.webp</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -31778,12 +31783,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Npc_molly</t>
+          <t>Church_guard</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>npc_molly_si_trial.png</t>
+          <t>church_guard_si_a.webp</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -31800,12 +31805,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Npc_robert</t>
+          <t>Church_guard</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>npc_robert_si_trial.png</t>
+          <t>church_guard_si_b.webp</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -31822,12 +31827,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Church_guard</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>aaron_si_angry.webp</t>
+          <t>church_guard_si_c.webp</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -31844,12 +31849,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Church_guard</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>aaron_si_armscross.webp</t>
+          <t>church_guard_si_d.webp</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -31866,12 +31871,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Church_guard</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>aaron_si_attention.webp</t>
+          <t>church_guard_si_e.webp</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -31888,12 +31893,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Church_guard</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>aaron_si_blindeye.webp</t>
+          <t>church_guard_si_f.webp</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -31910,12 +31915,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>f734e7ba-e7bb-457b-8cf7-66e13324c45d</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>aaron_si_closedsmile.webp</t>
+          <t>f734e7ba-e7bb-457b-8cf7-66e13324c45d.png</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -31932,12 +31937,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>aaron_si_confused.webp</t>
+          <t>mage_si_cast.webp</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -31954,12 +31959,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>aaron_si_draw.webp</t>
+          <t>molly_si_ask.webp</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -31976,12 +31981,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>aaron_si_front.webp</t>
+          <t>molly_si_closedtalk.webp</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -31998,12 +32003,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>aaron_si_signal.webp</t>
+          <t>molly_si_eyesmile.webp</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -32020,12 +32025,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Church_guard</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>church_guard_si_a.webp</t>
+          <t>molly_si_front.webp</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -32042,12 +32047,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Church_guard</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>church_guard_si_b.webp</t>
+          <t>molly_si_gossip.webp</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -32064,12 +32069,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Church_guard</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>church_guard_si_c.webp</t>
+          <t>molly_si_lookdown.webp</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -32086,12 +32091,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Church_guard</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>church_guard_si_d.webp</t>
+          <t>molly_si_order.webp</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -32108,12 +32113,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Church_guard</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>church_guard_si_e.webp</t>
+          <t>molly_si_serious.webp</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -32130,12 +32135,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Church_guard</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>church_guard_si_f.webp</t>
+          <t>molly_si_softsmile.webp</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -32152,12 +32157,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>f734e7ba-e7bb-457b-8cf7-66e13324c45d</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>f734e7ba-e7bb-457b-8cf7-66e13324c45d.png</t>
+          <t>molly_si_stern.webp</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -32174,12 +32179,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>mage_si_cast.webp</t>
+          <t>molly_si_superior.webp</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -32196,12 +32201,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Molly</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>mage_si_hurtsmile.webp</t>
+          <t>molly_si_surprise.webp</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -32223,7 +32228,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>molly_si_ask.webp</t>
+          <t>molly_si_talk.webp</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -32245,7 +32250,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>molly_si_closedtalk.webp</t>
+          <t>molly_si_think.webp</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -32267,7 +32272,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>molly_si_eyesmile.webp</t>
+          <t>molly_si_whisper.webp</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -32284,12 +32289,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>npc_ss_lofa_shoot</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>molly_si_front.webp</t>
+          <t>npc_ss_lofa_shoot.png</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -32306,12 +32311,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>molly_si_gossip.webp</t>
+          <t>robert_si_blindeye.webp</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -32328,12 +32333,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>molly_si_lookdown.webp</t>
+          <t>robert_si_bow.webp</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -32350,12 +32355,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>molly_si_order.webp</t>
+          <t>robert_si_closedtalk.webp</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -32372,12 +32377,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>molly_si_serious.webp</t>
+          <t>robert_si_front.webp</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -32394,12 +32399,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>molly_si_softsmile.webp</t>
+          <t>robert_si_sideeye.webp</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -32416,12 +32421,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>molly_si_stern.webp</t>
+          <t>robert_si_surprise.webp</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -32438,12 +32443,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>molly_si_superior.webp</t>
+          <t>robert_si_talk.webp</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -32460,12 +32465,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>molly_si_surprise.webp</t>
+          <t>renna_si_evalutatingclosemouth.webp</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -32482,12 +32487,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>molly_si_talk.webp</t>
+          <t>renna_si_annoy.webp</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -32504,12 +32509,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>Sorana</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>molly_si_think.webp</t>
+          <t>sorana_si_q.webp</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -32526,12 +32531,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Molly</t>
+          <t>image - 2026-09-20T150615.066</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>molly_si_whisper.webp</t>
+          <t>image - 2026-09-20T150615.066.png</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -32548,12 +32553,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>npc_ss_lofa_shoot</t>
+          <t>image - 2026-09-20T150842.343</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>npc_ss_lofa_shoot.png</t>
+          <t>image - 2026-09-20T150842.343.png</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -32570,12 +32575,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>image - 2026-09-20T151013.881</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>robert_si_blindeye.webp</t>
+          <t>image - 2026-09-20T151013.881.png</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -32592,12 +32597,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>image - 2026-09-20T151141.942</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>robert_si_bow.webp</t>
+          <t>image - 2026-09-20T151141.942.png</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -32614,12 +32619,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Torsten</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>robert_si_closedtalk.webp</t>
+          <t>torsten_si_front.webp</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -32636,12 +32641,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Torsten</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>robert_si_front.webp</t>
+          <t>torsten_si_q.webp</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -32658,12 +32663,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Xanya</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>robert_si_sideeye.webp</t>
+          <t>xanya_si_front.webp</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -32675,264 +32680,264 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Anya</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>robert_si_surprise.webp</t>
+          <t>resources/si/anya_si_nod.png</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 anya_si_nod.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>robert_si_talk.webp</t>
+          <t>resources/si/cecilie_si_saintinstall.png</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 cecilie_si_saintinstall.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Renna</t>
+          <t>Misha</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>renna_si_evalutatingclosemouth.webp</t>
+          <t>resources/si/misha_si_fight.png</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 misha_si_fight.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Renna</t>
+          <t>Misha</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>renna_si_annoy.webp</t>
+          <t>resources/si/misha_si_ni.png</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 misha_si_ni.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Sorana</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>sorana_si_q.webp</t>
+          <t>resources/si/nouvelle_si_gossip1.png</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 nouvelle_si_gossip1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T150615.066</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T150615.066.png</t>
+          <t>resources/si/nouvelle_si_salute.png</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 nouvelle_si_salute.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T150842.343</t>
+          <t>Nouvelle</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T150842.343.png</t>
+          <t>resources/si/nouvelle_si_sigh.png</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 nouvelle_si_sigh.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T151013.881</t>
+          <t>Npc_grocer</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T151013.881.png</t>
+          <t>resources/si/npc/npc_grocer_si_v2.webp</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T151141.942</t>
+          <t>Npc_grocer</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>image - 2026-09-20T151141.942.png</t>
+          <t>resources/si/npc/npc_grocer_si_v3.webp</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Torsten</t>
+          <t>Npc_grocer</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>torsten_si_front.webp</t>
+          <t>resources/si/npc/npc_grocer_si_v4.webp</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Torsten</t>
+          <t>Npc_grocer</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>torsten_si_q.webp</t>
+          <t>resources/si/npc/npc_grocer_si_v5.webp</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>美術交了沒接線</t>
+          <t>同差分的另一個版本</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Xanya</t>
+          <t>Npc_guildcounter</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>xanya_si_front.webp</t>
+          <t>resources/si/npc/npc_guildcounter_si_v1.webp</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>在 script/speakers.js 的 ART 補一筆 expr，並量 fx／top／bot（§6.5）</t>
+          <t>線上跑的是 npc_guildcounter_si_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -32944,17 +32949,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Anya</t>
+          <t>Npc_guildcounter</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>resources/si/anya_si_nod.png</t>
+          <t>resources/si/npc/npc_guildcounter_si_v3.webp</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>線上跑的是 anya_si_nod.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 npc_guildcounter_si_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -32966,17 +32971,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Npc_guildcounter</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>resources/si/cecilie_si_saintinstall.png</t>
+          <t>resources/si/npc/npc_guildcounter_si_v4.webp</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>線上跑的是 cecilie_si_saintinstall.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 npc_guildcounter_si_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -32988,17 +32993,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Misha</t>
+          <t>Npc_gunsmith</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>resources/si/misha_si_fight.png</t>
+          <t>resources/si/npc/npc_gunsmith_si_v2.webp</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>線上跑的是 misha_si_fight.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33010,17 +33015,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Misha</t>
+          <t>Npc_gunsmith</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>resources/si/misha_si_ni.png</t>
+          <t>resources/si/npc/npc_gunsmith_si_v3.webp</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>線上跑的是 misha_si_ni.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33032,17 +33037,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Npc_gunsmith</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>resources/si/nouvelle_si_gossip1.png</t>
+          <t>resources/si/npc/npc_gunsmith_si_v4.webp</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>線上跑的是 nouvelle_si_gossip1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33054,17 +33059,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Npc_gunsmith</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>resources/si/nouvelle_si_salute.png</t>
+          <t>resources/si/npc/npc_gunsmith_si_v5.webp</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>線上跑的是 nouvelle_si_salute.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33076,17 +33081,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Nouvelle</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>resources/si/nouvelle_si_sigh.png</t>
+          <t>resources/si/old/cecilie_si_front.png</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>線上跑的是 nouvelle_si_sigh.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 cecilie_si_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33098,17 +33103,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Npc_grocer</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_grocer_si_v2.webp</t>
+          <t>resources/si/old/cecilie_si_lookaside.png</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 cecilie_si_lookaside.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33120,17 +33125,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Npc_grocer</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_grocer_si_v3.webp</t>
+          <t>resources/si/old/cecilie_si_sadback.png</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 cecilie_si_sadback.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33142,17 +33147,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Npc_grocer</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_grocer_si_v4.webp</t>
+          <t>resources/si/old/cecilie_si_smile.png</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 cecilie_si_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33164,17 +33169,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Npc_grocer</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_grocer_si_v5.webp</t>
+          <t>resources/si/old/cecilie_si_tease.png</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_grocer_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 cecilie_si_tease.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33186,17 +33191,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Npc_guildcounter</t>
+          <t>Cecilie</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_guildcounter_si_v1.webp</t>
+          <t>resources/si/old/cecilie_si_upset.png</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_guildcounter_si_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 cecilie_si_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33208,17 +33213,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Npc_guildcounter</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_guildcounter_si_v3.webp</t>
+          <t>resources/si/renna_newhair/renna_si_argue.webp</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_guildcounter_si_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_argue.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33230,17 +33235,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Npc_guildcounter</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_guildcounter_si_v4.webp</t>
+          <t>resources/si/renna_newhair/renna_si_arguecute.webp</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_guildcounter_si_v5.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_arguecute.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33252,17 +33257,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Npc_gunsmith</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_gunsmith_si_v2.webp</t>
+          <t>resources/si/renna_newhair/renna_si_ask.webp</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_ask.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33274,17 +33279,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Npc_gunsmith</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_gunsmith_si_v3.webp</t>
+          <t>resources/si/renna_newhair/renna_si_askserious.webp</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_askserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33296,17 +33301,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Npc_gunsmith</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_gunsmith_si_v4.webp</t>
+          <t>resources/si/renna_newhair/renna_si_awkwerd.webp</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_awkwerd.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33318,17 +33323,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Npc_gunsmith</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>resources/si/npc/npc_gunsmith_si_v5.webp</t>
+          <t>resources/si/renna_newhair/renna_si_blush.webp</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>線上跑的是 npc_gunsmith_si_v1.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_blush.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33340,17 +33345,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>resources/si/old/cecilie_si_front.png</t>
+          <t>resources/si/renna_newhair/renna_si_bow.webp</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>線上跑的是 cecilie_si_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_bow.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33362,17 +33367,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>resources/si/old/cecilie_si_lookaside.png</t>
+          <t>resources/si/renna_newhair/renna_si_callangry.webp</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>線上跑的是 cecilie_si_lookaside.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_callangry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33384,17 +33389,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>resources/si/old/cecilie_si_sadback.png</t>
+          <t>resources/si/renna_newhair/renna_si_chase.webp</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>線上跑的是 cecilie_si_sadback.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_chase.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33406,17 +33411,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>resources/si/old/cecilie_si_smile.png</t>
+          <t>resources/si/renna_newhair/renna_si_chase2.webp</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>線上跑的是 cecilie_si_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_chase2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33428,17 +33433,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>resources/si/old/cecilie_si_tease.png</t>
+          <t>resources/si/renna_newhair/renna_si_command.webp</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>線上跑的是 cecilie_si_tease.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_command.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33450,17 +33455,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Cecilie</t>
+          <t>Renna</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>resources/si/old/cecilie_si_upset.png</t>
+          <t>resources/si/renna_newhair/renna_si_covermouth.webp</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>線上跑的是 cecilie_si_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_covermouth.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33477,12 +33482,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_argue.webp</t>
+          <t>resources/si/renna_newhair/renna_si_cringe.webp</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_argue.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_cringe.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33499,12 +33504,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_arguecute.webp</t>
+          <t>resources/si/renna_newhair/renna_si_curious.webp</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_arguecute.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_curious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33521,12 +33526,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_ask.webp</t>
+          <t>resources/si/renna_newhair/renna_si_die.webp</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_ask.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_die.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33543,12 +33548,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_askserious.webp</t>
+          <t>resources/si/renna_newhair/renna_si_evaluate.webp</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_askserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_evaluate.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33565,12 +33570,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_awkwerd.webp</t>
+          <t>resources/si/renna_newhair/renna_si_front.webp</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_awkwerd.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33587,12 +33592,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_blush.webp</t>
+          <t>resources/si/renna_newhair/renna_si_intense.webp</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_blush.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_intense.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33609,12 +33614,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_bow.webp</t>
+          <t>resources/si/renna_newhair/renna_si_intense2.webp</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_bow.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_intense2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33631,12 +33636,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_callangry.webp</t>
+          <t>resources/si/renna_newhair/renna_si_invite.webp</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_callangry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_invite.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33653,12 +33658,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_chase.webp</t>
+          <t>resources/si/renna_newhair/renna_si_lookaway.webp</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_chase.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_lookaway.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33675,12 +33680,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_chase2.webp</t>
+          <t>resources/si/renna_newhair/renna_si_lookawaytalk.webp</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_chase2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_lookawaytalk.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33697,12 +33702,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_command.webp</t>
+          <t>resources/si/renna_newhair/renna_si_lookdown.webp</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_command.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_lookdown.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33719,12 +33724,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_covermouth.webp</t>
+          <t>resources/si/renna_newhair/renna_si_lookup.webp</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_covermouth.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_lookup.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33741,12 +33746,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_cringe.webp</t>
+          <t>resources/si/renna_newhair/renna_si_pause.webp</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_cringe.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_pause.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33763,12 +33768,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_curious.webp</t>
+          <t>resources/si/renna_newhair/renna_si_relief.webp</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_curious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_relief.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33785,12 +33790,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_die.webp</t>
+          <t>resources/si/renna_newhair/renna_si_sad.webp</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_die.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_sad.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33807,12 +33812,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_evaluate.webp</t>
+          <t>resources/si/renna_newhair/renna_si_shout.webp</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_evaluate.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_shout.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33829,12 +33834,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_front.webp</t>
+          <t>resources/si/renna_newhair/renna_si_smile.webp</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_front.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33851,12 +33856,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_intense.webp</t>
+          <t>resources/si/renna_newhair/renna_si_stare.webp</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_intense.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_stare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33873,12 +33878,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_intense2.webp</t>
+          <t>resources/si/renna_newhair/renna_si_surprise.webp</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_intense2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_surprise.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33895,12 +33900,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_invite.webp</t>
+          <t>resources/si/renna_newhair/renna_si_talkserious.webp</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_invite.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_talkserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33917,12 +33922,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_lookaway.webp</t>
+          <t>resources/si/renna_newhair/renna_si_talkwork.webp</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_lookaway.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_talkwork.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33939,12 +33944,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_lookawaytalk.webp</t>
+          <t>resources/si/renna_newhair/renna_si_think.webp</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_lookawaytalk.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_think.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33961,12 +33966,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_lookdown.webp</t>
+          <t>resources/si/renna_newhair/renna_si_tire.webp</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_lookdown.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_tire.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -33983,12 +33988,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_lookup.webp</t>
+          <t>resources/si/renna_newhair/renna_si_upset.webp</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_lookup.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34005,12 +34010,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_pause.webp</t>
+          <t>resources/si/renna_newhair/renna_si_upsetstare.webp</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_pause.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_upsetstare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34027,12 +34032,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_relief.webp</t>
+          <t>resources/si/renna_newhair/renna_si_wake.webp</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_relief.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_wake.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34049,12 +34054,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_sad.webp</t>
+          <t>resources/si/renna_newhair/renna_si_watch.webp</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_sad.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_watch.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34071,12 +34076,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_shout.webp</t>
+          <t>resources/si/renna_newhair/renna_si_worry.webp</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_shout.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_worry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34093,12 +34098,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_smile.webp</t>
+          <t>resources/si/renna_newhair/renna_si_write.webp</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_smile.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_write.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34115,12 +34120,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_stare.webp</t>
+          <t>resources/si/renna_si_hug.png</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_stare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_hug.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34137,12 +34142,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_surprise.webp</t>
+          <t>resources/si/renna_si_hugangry2.png</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_surprise.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_hugangry2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34159,12 +34164,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_talkserious.webp</t>
+          <t>resources/si/renna_si_hugclose.png</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_talkserious.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_hugclose.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34181,12 +34186,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_talkwork.webp</t>
+          <t>resources/si/renna_si_huglookaway.png</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>線上跑的是 renna_si_talkwork.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
+          <t>線上跑的是 renna_si_huglookaway.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
       </c>
     </row>
@@ -34198,279 +34203,15 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Renna</t>
+          <t>Torsten</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>resources/si/renna_newhair/renna_si_think.webp</t>
+          <t>resources/si/torsten_si_back.png</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_think.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>resources/si/renna_newhair/renna_si_tire.webp</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_tire.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>resources/si/renna_newhair/renna_si_upset.webp</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_upset.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>resources/si/renna_newhair/renna_si_upsetstare.webp</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_upsetstare.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>resources/si/renna_newhair/renna_si_wake.webp</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_wake.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>resources/si/renna_newhair/renna_si_watch.webp</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_watch.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>resources/si/renna_newhair/renna_si_worry.webp</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_worry.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>resources/si/renna_newhair/renna_si_write.webp</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_write.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>resources/si/renna_si_hug.png</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_hug.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>resources/si/renna_si_hugangry2.png</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_hugangry2.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>resources/si/renna_si_hugclose.png</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_hugclose.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>Renna</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>resources/si/renna_si_huglookaway.png</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>線上跑的是 renna_si_huglookaway.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>同差分的另一個版本</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>Torsten</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>resources/si/torsten_si_back.png</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
         <is>
           <t>線上跑的是 torsten_si_back.webp —— 要換上去就改 speakers.js 的 src，並**重量** fx／top／bot（§5：換圖一定要重量取景）</t>
         </is>
@@ -41444,42 +41185,47 @@
       </c>
     </row>
     <row r="3" ht="111" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_battlecry.webp</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>battlecry</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>1528</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_battlecry.webp</t>
         </is>
@@ -41533,84 +41279,94 @@
       </c>
     </row>
     <row r="5" ht="111" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_call.webp</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>call</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1526</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_call.webp</t>
         </is>
       </c>
     </row>
     <row r="6" ht="111" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_command.webp</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="n"/>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>command</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>1526</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_command.webp</t>
         </is>
@@ -41860,168 +41616,188 @@
       </c>
     </row>
     <row r="12" ht="111" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_nosebleed.webp</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>nosebleed</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.553</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>1511</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_nosebleed.webp</t>
         </is>
       </c>
     </row>
     <row r="13" ht="111" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_pant.webp</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>pant</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>1443</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_pant.webp</t>
         </is>
       </c>
     </row>
     <row r="14" ht="111" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_proud.webp</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>proud</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>1526</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_proud.webp</t>
         </is>
       </c>
     </row>
     <row r="15" ht="111" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_ready.webp</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>1509</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_ready.webp</t>
         </is>
@@ -42130,126 +41906,141 @@
       </c>
     </row>
     <row r="18" ht="111" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_shocknose.webp</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>shocknose</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.401</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>1497</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_shocknose.webp</t>
         </is>
       </c>
     </row>
     <row r="19" ht="111" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_shyhand.webp</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>shyhand</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.5590000000000001</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>1498</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_shyhand.webp</t>
         </is>
       </c>
     </row>
     <row r="20" ht="111" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_shynose.webp</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>shynose</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>1496</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_shynose.webp</t>
         </is>
@@ -42307,42 +42098,47 @@
       </c>
     </row>
     <row r="22" ht="111" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>賽西莉</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>cecilie_si_smirk.webp</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>✘ 未接線</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>估</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>1024×1536</t>
-        </is>
-      </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>smirk</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>1529</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>1024×1536</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>resources/si/cecilie_si_smirk.webp</t>
         </is>

</xml_diff>